<commit_message>
feat: locate unambiguous native PDF evidence
</commit_message>
<xml_diff>
--- a/winwatt_automation/data/e2e/delceg_approved_project.xlsx
+++ b/winwatt_automation/data/e2e/delceg_approved_project.xlsx
@@ -15449,7 +15449,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -15460,13 +15460,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>(1497.19, 254.13, 1594.76, 265.47)</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -15647,7 +15652,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -15658,13 +15663,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>(1430.01, 585.22, 1494.81, 596.56)</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -16687,7 +16697,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>É-02C</t>
+          <t>..\test\É02C_TERVEZETT PINCESZINTI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -16698,13 +16708,18 @@
           <t>É-02C</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>(409.74, 478.5, 424.87, 487.17)</t>
+        </is>
+      </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>spreadsheet_import:A 'lpcsh.' / beton / 2,21 m² bélyegből; rövidítés feloldása értelmezés, ezért je</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q26" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -17017,7 +17032,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -17028,13 +17043,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>(1156.54, 117.84, 1273.4, 129.18)</t>
+        </is>
+      </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -17555,7 +17575,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -17566,13 +17586,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>(1424.26, 448.02, 1527.08, 459.36)</t>
+        </is>
+      </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q39" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -18027,7 +18052,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -18038,13 +18063,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>(341.68, 429.58, 360.81, 438.26)</t>
+        </is>
+      </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q46" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S46" t="inlineStr">
         <is>
@@ -18349,7 +18379,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M51" t="n">
@@ -18360,13 +18390,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>(1156.54, 526.03, 1257.37, 537.37)</t>
+        </is>
+      </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -20303,7 +20338,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M80" t="n">
@@ -20314,13 +20349,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>(1163.66, 560.05, 1243.95, 571.38)</t>
+        </is>
+      </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q80" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S80" t="inlineStr">
         <is>
@@ -20572,7 +20612,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M84" t="n">
@@ -20583,13 +20623,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>(1430.01, 140.75, 1510.85, 152.08)</t>
+        </is>
+      </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q84" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S84" t="inlineStr">
         <is>
@@ -20988,7 +21033,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M90" t="n">
@@ -20999,13 +21044,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>(436.07, 709.66, 455.52, 718.33)</t>
+        </is>
+      </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q90" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S90" t="inlineStr">
         <is>
@@ -21054,7 +21104,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M91" t="n">
@@ -21065,13 +21115,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>(1156.54, 537.37, 1264.98, 548.71)</t>
+        </is>
+      </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q91" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S91" t="inlineStr">
         <is>
@@ -21120,7 +21175,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M92" t="n">
@@ -21131,13 +21186,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>(1154.44, 503.35, 1261.93, 514.69)</t>
+        </is>
+      </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q92" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S92" t="inlineStr">
         <is>
@@ -21521,7 +21581,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M98" t="n">
@@ -21532,13 +21592,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>(1168.77, 548.71, 1246.98, 560.04)</t>
+        </is>
+      </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q98" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S98" t="inlineStr">
         <is>
@@ -22480,7 +22545,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>É-02C + É-03</t>
+          <t>..\test\É02C_TERVEZETT PINCESZINTI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M112" t="n">
@@ -22491,13 +22556,18 @@
           <t>É-02C + É-03</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>(409.74, 478.5, 424.87, 487.17)</t>
+        </is>
+      </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>spreadsheet_import:A 2,21 m²-es lépcsőházi bélyeg és a pincei pozíció alapján.</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q112" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S112" t="inlineStr">
         <is>
@@ -22759,7 +22829,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>É-02C + É-03</t>
+          <t>..\test\É02C_TERVEZETT PINCESZINTI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M116" t="n">
@@ -22770,13 +22840,18 @@
           <t>É-02C + É-03</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>(376.79, 348.42, 396.24, 357.1)</t>
+        </is>
+      </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>spreadsheet_import:Helyiségbélyeg 67,95 m²; É-03 R14 'Talajon fekvő padló'.</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q116" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S116" t="inlineStr">
         <is>
@@ -22962,7 +23037,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M119" t="n">
@@ -22973,13 +23048,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>(1129.72, 673.43, 1167.39, 684.77)</t>
+        </is>
+      </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q119" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -23576,7 +23656,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>É-02C</t>
+          <t>..\test\É02C_TERVEZETT PINCESZINTI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M128" t="n">
@@ -23587,13 +23667,18 @@
           <t>É-02C</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>(376.79, 348.42, 396.24, 357.1)</t>
+        </is>
+      </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>spreadsheet_import:A pince alaprajz központi helyiségbélyegéből: PINCE / beton / 67,95 m².</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q128" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
@@ -24530,7 +24615,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M142" t="n">
@@ -24541,13 +24626,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>(468.22, 659.68, 483.35, 668.36)</t>
+        </is>
+      </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q142" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -24596,7 +24686,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M143" t="n">
@@ -24607,13 +24697,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>(1399.54, 737.16, 1510.98, 748.49)</t>
+        </is>
+      </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q143" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S143" t="inlineStr">
         <is>
@@ -25200,7 +25295,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M152" t="n">
@@ -25211,13 +25306,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>(342.83, 731.26, 362.29, 739.94)</t>
+        </is>
+      </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q152" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S152" t="inlineStr">
         <is>
@@ -26484,7 +26584,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M171" t="n">
@@ -26495,13 +26595,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>(317.18, 582.48, 336.64, 591.15)</t>
+        </is>
+      </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q171" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S171" t="inlineStr">
         <is>
@@ -28113,7 +28218,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M195" t="n">
@@ -28124,13 +28229,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>(1426.36, 186.1, 1520.69, 197.44)</t>
+        </is>
+      </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q195" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S195" t="inlineStr">
         <is>
@@ -28585,7 +28695,7 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M202" t="n">
@@ -28596,13 +28706,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>(1426.36, 129.41, 1522.87, 140.74)</t>
+        </is>
+      </c>
       <c r="P202" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q202" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S202" t="inlineStr">
         <is>
@@ -29265,7 +29380,7 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M212" t="n">
@@ -29276,13 +29391,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>(424.49, 306.36, 443.94, 315.04)</t>
+        </is>
+      </c>
       <c r="P212" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q212" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S212" t="inlineStr">
         <is>
@@ -29747,7 +29867,7 @@
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M219" t="n">
@@ -29758,13 +29878,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>(1399.54, 118.07, 1496.72, 129.41)</t>
+        </is>
+      </c>
       <c r="P219" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q219" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S219" t="inlineStr">
         <is>
@@ -30219,7 +30344,7 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M226" t="n">
@@ -30230,13 +30355,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>(318.1, 332.89, 365.63, 341.57)</t>
+        </is>
+      </c>
       <c r="P226" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q226" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S226" t="inlineStr">
         <is>
@@ -30488,7 +30618,7 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M230" t="n">
@@ -30499,13 +30629,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>(1129.72, 560.05, 1144.65, 571.38)</t>
+        </is>
+      </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q230" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S230" t="inlineStr">
         <is>
@@ -31092,7 +31227,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M239" t="n">
@@ -31103,13 +31238,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>(1430.01, 572.75, 1559.78, 584.08)</t>
+        </is>
+      </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q239" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S239" t="inlineStr">
         <is>
@@ -32584,7 +32724,7 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M261" t="n">
@@ -32595,13 +32735,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>(1430.01, 242.79, 1503.6, 254.13)</t>
+        </is>
+      </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q261" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S261" t="inlineStr">
         <is>
@@ -33599,7 +33744,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M276" t="n">
@@ -33610,13 +33755,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>(276.36, 794.65, 339.09, 803.32)</t>
+        </is>
+      </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből; kültéri fa burkolat jelölve.</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q276" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S276" t="inlineStr">
         <is>
@@ -34010,7 +34160,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M282" t="n">
@@ -34021,13 +34171,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>(459.56, 558.88, 498.87, 567.55)</t>
+        </is>
+      </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q282" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S282" t="inlineStr">
         <is>
@@ -34147,7 +34302,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M284" t="n">
@@ -34158,13 +34313,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>(1129.72, 928.02, 1202.5, 939.36)</t>
+        </is>
+      </c>
       <c r="P284" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q284" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S284" t="inlineStr">
         <is>
@@ -34279,7 +34439,7 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M286" t="n">
@@ -34290,13 +34450,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>(1176.06, 163.19, 1209.81, 174.53)</t>
+        </is>
+      </c>
       <c r="P286" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q286" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S286" t="inlineStr">
         <is>
@@ -34482,7 +34647,7 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M289" t="n">
@@ -34493,13 +34658,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>(1156.54, 662.09, 1248.81, 673.43)</t>
+        </is>
+      </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q289" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S289" t="inlineStr">
         <is>
@@ -34619,7 +34789,7 @@
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M291" t="n">
@@ -34630,13 +34800,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>(276.36, 812.46, 291.49, 821.14)</t>
+        </is>
+      </c>
       <c r="P291" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből; kültéri fa burkolat jelölve.</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q291" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S291" t="inlineStr">
         <is>
@@ -34832,7 +35007,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M294" t="n">
@@ -34843,13 +35018,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>(318.1, 350.71, 337.23, 359.39)</t>
+        </is>
+      </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q294" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S294" t="inlineStr">
         <is>
@@ -35243,7 +35423,7 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M300" t="n">
@@ -35254,13 +35434,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>(1198.88, 140.52, 1284.03, 151.85)</t>
+        </is>
+      </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q300" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S300" t="inlineStr">
         <is>
@@ -35512,7 +35697,7 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M304" t="n">
@@ -35523,13 +35708,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>(1156.54, 140.52, 1284.03, 151.85)</t>
+        </is>
+      </c>
       <c r="P304" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q304" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S304" t="inlineStr">
         <is>
@@ -36192,7 +36382,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M314" t="n">
@@ -36203,13 +36393,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>(464.91, 400.75, 480.05, 409.43)</t>
+        </is>
+      </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>spreadsheet_import:A helyiségbélyegből: név + burkolat + m²; a 'bm.:1,90 m' és 'hasznos at.' felira</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q314" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S314" t="inlineStr">
         <is>
@@ -37131,7 +37326,7 @@
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t>É-02C + É-03</t>
+          <t>..\test\É02C_TERVEZETT PINCESZINTI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M328" t="n">
@@ -37142,13 +37337,18 @@
           <t>É-02C + É-03</t>
         </is>
       </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>(370.6, 222.56, 389.52, 233.41)</t>
+        </is>
+      </c>
       <c r="P328" t="inlineStr">
         <is>
-          <t>spreadsheet_import:É-02C belső hosszméret 9,49 m; É-03 A-A/C-C metszeten pince belmagasság környeze</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q328" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S328" t="inlineStr">
         <is>
@@ -37197,7 +37397,7 @@
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M329" t="n">
@@ -37208,13 +37408,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>(1399.54, 748.49, 1485.1, 759.83)</t>
+        </is>
+      </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q329" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S329" t="inlineStr">
         <is>
@@ -38354,7 +38559,7 @@
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M346" t="n">
@@ -38365,13 +38570,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O346" t="inlineStr">
+        <is>
+          <t>(467.17, 444.01, 482.3, 452.69)</t>
+        </is>
+      </c>
       <c r="P346" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q346" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S346" t="inlineStr">
         <is>
@@ -38953,7 +39163,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M355" t="n">
@@ -38964,13 +39174,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O355" t="inlineStr">
+        <is>
+          <t>(1430.01, 633.97, 1505.87, 645.31)</t>
+        </is>
+      </c>
       <c r="P355" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q355" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S355" t="inlineStr">
         <is>
@@ -39019,7 +39234,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M356" t="n">
@@ -39030,13 +39245,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O356" t="inlineStr">
+        <is>
+          <t>(1156.54, 650.75, 1218.62, 662.09)</t>
+        </is>
+      </c>
       <c r="P356" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q356" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S356" t="inlineStr">
         <is>
@@ -39222,7 +39442,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M359" t="n">
@@ -39233,13 +39453,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O359" t="inlineStr">
+        <is>
+          <t>(1129.72, 916.68, 1203.4, 928.02)</t>
+        </is>
+      </c>
       <c r="P359" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q359" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S359" t="inlineStr">
         <is>
@@ -39430,7 +39655,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M362" t="n">
@@ -39441,13 +39666,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O362" t="inlineStr">
+        <is>
+          <t>(464.91, 382.94, 492.56, 391.61)</t>
+        </is>
+      </c>
       <c r="P362" t="inlineStr">
         <is>
-          <t>spreadsheet_import:A helyiségbélyegből: név + burkolat + m²; a 'bm.:1,90 m' és 'hasznos at.' felira</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q362" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S362" t="inlineStr">
         <is>
@@ -39699,7 +39929,7 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>É-03</t>
+          <t>..\test\É03_TERVEZETT METSZETEK_végl.pdf</t>
         </is>
       </c>
       <c r="M366" t="n">
@@ -39710,13 +39940,18 @@
           <t>É-03</t>
         </is>
       </c>
+      <c r="O366" t="inlineStr">
+        <is>
+          <t>(1154.44, 514.69, 1274.05, 526.03)</t>
+        </is>
+      </c>
       <c r="P366" t="inlineStr">
         <is>
-          <t>spreadsheet_import:spreadsheet_import</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q366" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S366" t="inlineStr">
         <is>
@@ -39902,7 +40137,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>É-02B</t>
+          <t>..\test\É02B_TERVEZETT TETŐTÉRI ALAPRAJZ_végl.pdf</t>
         </is>
       </c>
       <c r="M369" t="n">
@@ -39913,13 +40148,18 @@
           <t>É-02B</t>
         </is>
       </c>
+      <c r="O369" t="inlineStr">
+        <is>
+          <t>(459.56, 576.69, 474.69, 585.37)</t>
+        </is>
+      </c>
       <c r="P369" t="inlineStr">
         <is>
-          <t>spreadsheet_import:helyiségbélyegből</t>
+          <t>native_pdf_text_exact</t>
         </is>
       </c>
       <c r="Q369" t="n">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="S369" t="inlineStr">
         <is>

</xml_diff>